<commit_message>
Add RSVP status field to participant management
Introduce RSVP column to track participant response status (Yes/No). Changes include:
- New required 'rsvp' column in Excel roster import
- RSVP field in database schema with migration support
- UI filter and display in participant list (does not affect attendance/deck)
- Updated test data and validation
</commit_message>
<xml_diff>
--- a/tests/sample_data/participants.xlsx
+++ b/tests/sample_data/participants.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +449,11 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>RSVP</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Department</t>
         </is>
       </c>
@@ -486,6 +491,11 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>R&amp;D</t>
         </is>
       </c>
@@ -523,6 +533,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>R&amp;D</t>
         </is>
       </c>
@@ -560,6 +575,11 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>QA</t>
         </is>
       </c>
@@ -597,6 +617,11 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>Ops</t>
         </is>
       </c>
@@ -634,6 +659,11 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>Ops</t>
         </is>
       </c>
@@ -671,6 +701,11 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>Admin</t>
         </is>
       </c>
@@ -707,6 +742,11 @@
         </is>
       </c>
       <c r="G8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>

</xml_diff>